<commit_message>
Fichier d'exemple Pro : baisses de prix et nouvelles annonces alignées sur le site
- Colonne « Baisse de prix » : « Dès le 4e relevé » remplacé par « - » (le
  fichier vient du premier relevé, sans relevé précédent pour comparer).
- Feuille « Contenu » : « Nouvelle » = absente du relevé précédent, comme
  sur les pages villes ; sur cet exemple tiré du premier relevé, « Oui »
  signale une annonce publiée dans les 7 jours précédents. Baisse de prix =
  prix demandé en baisse depuis le relevé précédent.
- Les 20 annonces (titres, agences, prix, liens) ne changent pas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V6V9dHCPRkZdCTMnTwWbDp
</commit_message>
<xml_diff>
--- a/exemples/atlas-data-pro-exemple-gueliz.xlsx
+++ b/exemples/atlas-data-pro-exemple-gueliz.xlsx
@@ -588,7 +588,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Dès le 4e relevé</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M2" s="5" t="inlineStr">
@@ -641,7 +641,7 @@
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Dès le 4e relevé</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M3" s="5" t="inlineStr">
@@ -694,7 +694,7 @@
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Dès le 4e relevé</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M4" s="5" t="inlineStr">
@@ -747,7 +747,7 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Dès le 4e relevé</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M5" s="5" t="inlineStr">
@@ -800,7 +800,7 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Dès le 4e relevé</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M6" s="5" t="inlineStr">
@@ -853,7 +853,7 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Dès le 4e relevé</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M7" s="5" t="inlineStr">
@@ -906,7 +906,7 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Dès le 4e relevé</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M8" s="5" t="inlineStr">
@@ -959,7 +959,7 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Dès le 4e relevé</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M9" s="5" t="inlineStr">
@@ -1012,7 +1012,7 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Dès le 4e relevé</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M10" s="5" t="inlineStr">
@@ -1065,7 +1065,7 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Dès le 4e relevé</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M11" s="5" t="inlineStr">
@@ -1118,7 +1118,7 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Dès le 4e relevé</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M12" s="5" t="inlineStr">
@@ -1171,7 +1171,7 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Dès le 4e relevé</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M13" s="5" t="inlineStr">
@@ -1224,7 +1224,7 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Dès le 4e relevé</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M14" s="5" t="inlineStr">
@@ -1277,7 +1277,7 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Dès le 4e relevé</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M15" s="5" t="inlineStr">
@@ -1330,7 +1330,7 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Dès le 4e relevé</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M16" s="5" t="inlineStr">
@@ -1383,7 +1383,7 @@
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Dès le 4e relevé</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M17" s="5" t="inlineStr">
@@ -1436,7 +1436,7 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Dès le 4e relevé</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M18" s="5" t="inlineStr">
@@ -1489,7 +1489,7 @@
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Dès le 4e relevé</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M19" s="5" t="inlineStr">
@@ -1542,7 +1542,7 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Dès le 4e relevé</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M20" s="5" t="inlineStr">
@@ -1595,7 +1595,7 @@
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Dès le 4e relevé</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M21" s="5" t="inlineStr">
@@ -1696,7 +1696,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>« Oui » si l’annonce a été publiée dans les 7 jours précédant le relevé (lignes surlignées).</t>
+          <t>« Oui » si l’annonce n’était pas dans le relevé précédent. Ce fichier d’exemple vient du premier relevé (17 octobre 2026) : « Oui » y signale une annonce publiée dans les 7 jours précédant le relevé (lignes surlignées).</t>
         </is>
       </c>
     </row>
@@ -1708,7 +1708,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Calculée en comparant les relevés hebdomadaires successifs, disponible dès le 4e relevé.</t>
+          <t>« Oui » si le prix demandé a baissé depuis le relevé précédent. Ce fichier d’exemple vient du premier relevé : la colonne y est vide (-).</t>
         </is>
       </c>
     </row>

</xml_diff>